<commit_message>
Implementation of Task 2.1 of Stripe and Subscription integration. Necesseray refactorings in the api gateway for the endpoints, the checkout controller, the token controller, database access files and payment, subscription and stripe service. Seed files improvement for pricing information. Documentation addition for planning and pricing. Recalculation of pricing. Development of frontend components for pricing, checkout buttons and pages
</commit_message>
<xml_diff>
--- a/docs/content/docs/7_pricing/2_subscriptiontoken_calculator.xlsx
+++ b/docs/content/docs/7_pricing/2_subscriptiontoken_calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Short-Video-Creator-Simplified\docs\content\docs\7_pricing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94CE31BE-C208-4741-AD79-E3E7B507074A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D080A330-F014-47E1-B19F-CE17D5966B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="797" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="797" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Services" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,14 @@
     <sheet name="IAM AuthO" sheetId="10" r:id="rId3"/>
     <sheet name="LLM" sheetId="2" r:id="rId4"/>
     <sheet name="Image" sheetId="4" r:id="rId5"/>
-    <sheet name="Voice" sheetId="3" r:id="rId6"/>
-    <sheet name="Animation" sheetId="6" r:id="rId7"/>
-    <sheet name="Video" sheetId="7" r:id="rId8"/>
-    <sheet name="Music" sheetId="5" r:id="rId9"/>
-    <sheet name="Assembly" sheetId="8" r:id="rId10"/>
+    <sheet name="Image (AceData)" sheetId="11" r:id="rId6"/>
+    <sheet name="Voice" sheetId="3" r:id="rId7"/>
+    <sheet name="Animation" sheetId="6" r:id="rId8"/>
+    <sheet name="Video" sheetId="7" r:id="rId9"/>
+    <sheet name="Music (AceData)" sheetId="5" r:id="rId10"/>
+    <sheet name="Assembly" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="249">
   <si>
     <t>Image</t>
   </si>
@@ -1302,6 +1302,9 @@
   </si>
   <si>
     <t>Information: For calculation of the service overview we considered for each service the most expensive package. Depending on traffic, user amount and usage we can select a different package and also increase monthly payment to yearly payment (when the software is succesful) which would decrease the cost for each service. This should be considered in pricing.</t>
+  </si>
+  <si>
+    <t>Information Ace Data: 2.7945 Credits (fast) is one image; 5.589 Credits / Call for turbo</t>
   </si>
 </sst>
 </file>
@@ -1479,7 +1482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1546,6 +1549,9 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1591,6 +1597,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1900,31 +1907,31 @@
       <c r="B1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="29" t="s">
         <v>241</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28" t="s">
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="28" t="s">
+      <c r="J1" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28" t="s">
+      <c r="K1" s="29"/>
+      <c r="L1" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28" t="s">
+      <c r="M1" s="29"/>
+      <c r="N1" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="O1" s="28"/>
+      <c r="O1" s="29"/>
     </row>
     <row r="2" spans="1:15" s="1" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="C2" s="1" t="s">
@@ -2010,11 +2017,11 @@
         <v>0.79360000000000008</v>
       </c>
       <c r="L3" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M3" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N3" s="2">
@@ -2071,11 +2078,11 @@
         <v>1.5872000000000002</v>
       </c>
       <c r="L4" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M4" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N4" s="2">
@@ -2132,11 +2139,11 @@
         <v>2.3808000000000002</v>
       </c>
       <c r="L5" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M5" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N5" s="2">
@@ -2193,11 +2200,11 @@
         <v>3.1744000000000003</v>
       </c>
       <c r="L6" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M6" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N6" s="2">
@@ -2254,11 +2261,11 @@
         <v>3.9680000000000004</v>
       </c>
       <c r="L7" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M7" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N7" s="2">
@@ -2315,11 +2322,11 @@
         <v>4.7616000000000005</v>
       </c>
       <c r="L8" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M8" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N8" s="2">
@@ -2376,11 +2383,11 @@
         <v>5.555200000000001</v>
       </c>
       <c r="L9" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M9" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N9" s="2">
@@ -2437,11 +2444,11 @@
         <v>6.3488000000000007</v>
       </c>
       <c r="L10" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M10" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N10" s="2">
@@ -2498,11 +2505,11 @@
         <v>7.1424000000000003</v>
       </c>
       <c r="L11" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M11" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N11" s="2">
@@ -2559,11 +2566,11 @@
         <v>7.9360000000000008</v>
       </c>
       <c r="L12" s="7">
-        <f>Music!$F$24</f>
+        <f>'Music (AceData)'!$F$24</f>
         <v>5.7236363636363634E-2</v>
       </c>
       <c r="M12" s="2">
-        <f>Music!$F$26</f>
+        <f>'Music (AceData)'!$F$26</f>
         <v>6.123636363636363E-2</v>
       </c>
       <c r="N12" s="2">
@@ -2580,14 +2587,14 @@
       <c r="A14" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="I14" s="29" t="s">
+      <c r="I14" s="30" t="s">
         <v>247</v>
       </c>
-      <c r="J14" s="30"/>
-      <c r="K14" s="30"/>
-      <c r="L14" s="30"/>
-      <c r="M14" s="30"/>
-      <c r="N14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="32"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -2596,12 +2603,12 @@
       <c r="B15">
         <v>21</v>
       </c>
-      <c r="I15" s="32"/>
-      <c r="J15" s="33"/>
-      <c r="K15" s="33"/>
-      <c r="L15" s="33"/>
-      <c r="M15" s="33"/>
-      <c r="N15" s="34"/>
+      <c r="I15" s="33"/>
+      <c r="J15" s="34"/>
+      <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
+      <c r="M15" s="34"/>
+      <c r="N15" s="35"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -2610,12 +2617,12 @@
       <c r="B16">
         <v>6</v>
       </c>
-      <c r="I16" s="32"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="33"/>
-      <c r="L16" s="33"/>
-      <c r="M16" s="33"/>
-      <c r="N16" s="34"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="34"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="34"/>
+      <c r="M16" s="34"/>
+      <c r="N16" s="35"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -2624,12 +2631,12 @@
       <c r="B17">
         <v>20</v>
       </c>
-      <c r="I17" s="32"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-      <c r="L17" s="33"/>
-      <c r="M17" s="33"/>
-      <c r="N17" s="34"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
+      <c r="M17" s="34"/>
+      <c r="N17" s="35"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -2638,12 +2645,12 @@
       <c r="B18">
         <v>6</v>
       </c>
-      <c r="I18" s="32"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
-      <c r="L18" s="33"/>
-      <c r="M18" s="33"/>
-      <c r="N18" s="34"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="34"/>
+      <c r="L18" s="34"/>
+      <c r="M18" s="34"/>
+      <c r="N18" s="35"/>
     </row>
     <row r="19" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
@@ -2652,12 +2659,12 @@
       <c r="B19">
         <v>5</v>
       </c>
-      <c r="I19" s="35"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
-      <c r="L19" s="36"/>
-      <c r="M19" s="36"/>
-      <c r="N19" s="37"/>
+      <c r="I19" s="36"/>
+      <c r="J19" s="37"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="37"/>
+      <c r="M19" s="37"/>
+      <c r="N19" s="38"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -3319,6 +3326,476 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31193713-3E89-4A71-A172-6D7922B9768D}">
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="17.08984375" customWidth="1"/>
+    <col min="5" max="5" width="22.26953125" customWidth="1"/>
+    <col min="6" max="6" width="25.36328125" customWidth="1"/>
+    <col min="7" max="7" width="19.54296875" customWidth="1"/>
+    <col min="8" max="8" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>50</v>
+      </c>
+      <c r="E2">
+        <f>B2/D2</f>
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <f>C2/D2</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <f>E2*100</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <f>F2*100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <v>96</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>2500</v>
+      </c>
+      <c r="E3">
+        <f>B3/(D3*12)</f>
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="F3">
+        <f>C3/D3</f>
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="G3" s="2">
+        <f>E3*5</f>
+        <v>1.6E-2</v>
+      </c>
+      <c r="H3" s="2">
+        <f>F3*5</f>
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4">
+        <v>288</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
+      <c r="D4">
+        <v>10000</v>
+      </c>
+      <c r="E4">
+        <f>B4/(D4*12)</f>
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="F4">
+        <f t="shared" ref="F4" si="0">C4/D4</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="G4" s="2">
+        <f>E4*5</f>
+        <v>1.1999999999999999E-2</v>
+      </c>
+      <c r="H4" s="2">
+        <f>F4*5</f>
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11">
+        <v>13</v>
+      </c>
+      <c r="D11">
+        <v>100</v>
+      </c>
+      <c r="E11" s="43">
+        <f t="shared" ref="E11:E18" si="1">C11/D11</f>
+        <v>0.13</v>
+      </c>
+      <c r="F11" s="43"/>
+      <c r="G11" s="41">
+        <f>E11*$F$20</f>
+        <v>4.6800000000000001E-2</v>
+      </c>
+      <c r="H11" s="41"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12">
+        <v>63.2</v>
+      </c>
+      <c r="D12">
+        <v>530</v>
+      </c>
+      <c r="E12" s="43">
+        <f t="shared" si="1"/>
+        <v>0.11924528301886793</v>
+      </c>
+      <c r="F12" s="43"/>
+      <c r="G12" s="41">
+        <f t="shared" ref="G12:G18" si="2">E12*$F$20</f>
+        <v>4.2928301886792454E-2</v>
+      </c>
+      <c r="H12" s="41"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13">
+        <v>126</v>
+      </c>
+      <c r="D13">
+        <v>1100</v>
+      </c>
+      <c r="E13" s="43">
+        <f t="shared" si="1"/>
+        <v>0.11454545454545455</v>
+      </c>
+      <c r="F13" s="43"/>
+      <c r="G13" s="41">
+        <f t="shared" si="2"/>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="H13" s="41"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14">
+        <v>647</v>
+      </c>
+      <c r="D14">
+        <v>5950</v>
+      </c>
+      <c r="E14" s="43">
+        <f t="shared" si="1"/>
+        <v>0.10873949579831933</v>
+      </c>
+      <c r="F14" s="43"/>
+      <c r="G14" s="41">
+        <f t="shared" si="2"/>
+        <v>3.9146218487394961E-2</v>
+      </c>
+      <c r="H14" s="41"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15">
+        <v>1313</v>
+      </c>
+      <c r="D15">
+        <v>12500</v>
+      </c>
+      <c r="E15" s="43">
+        <f t="shared" si="1"/>
+        <v>0.10503999999999999</v>
+      </c>
+      <c r="F15" s="43"/>
+      <c r="G15" s="41">
+        <f t="shared" si="2"/>
+        <v>3.7814399999999998E-2</v>
+      </c>
+      <c r="H15" s="41"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16">
+        <v>2528</v>
+      </c>
+      <c r="D16">
+        <v>25000</v>
+      </c>
+      <c r="E16" s="43">
+        <f t="shared" si="1"/>
+        <v>0.10112</v>
+      </c>
+      <c r="F16" s="43"/>
+      <c r="G16" s="41">
+        <f t="shared" si="2"/>
+        <v>3.6403199999999997E-2</v>
+      </c>
+      <c r="H16" s="41"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17">
+        <v>6641</v>
+      </c>
+      <c r="D17">
+        <v>67500</v>
+      </c>
+      <c r="E17" s="43">
+        <f t="shared" si="1"/>
+        <v>9.8385185185185187E-2</v>
+      </c>
+      <c r="F17" s="43"/>
+      <c r="G17" s="41">
+        <f t="shared" si="2"/>
+        <v>3.5418666666666668E-2</v>
+      </c>
+      <c r="H17" s="41"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18">
+        <v>13584</v>
+      </c>
+      <c r="D18">
+        <v>142800</v>
+      </c>
+      <c r="E18" s="43">
+        <f t="shared" si="1"/>
+        <v>9.5126050420168071E-2</v>
+      </c>
+      <c r="F18" s="43"/>
+      <c r="G18" s="41">
+        <f t="shared" si="2"/>
+        <v>3.4245378151260504E-2</v>
+      </c>
+      <c r="H18" s="41"/>
+    </row>
+    <row r="20" spans="1:8" s="44" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" s="44">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A23" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="2">
+        <f>G3</f>
+        <v>1.6E-2</v>
+      </c>
+      <c r="E24" s="2">
+        <f>G13</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F24" s="2">
+        <f>D24+E24</f>
+        <v>5.7236363636363634E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="2">
+        <f>G4</f>
+        <v>1.1999999999999999E-2</v>
+      </c>
+      <c r="E25" s="2">
+        <f>G13</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F25" s="2">
+        <f t="shared" ref="F25:F27" si="3">D25+E25</f>
+        <v>5.323636363636363E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="2">
+        <f>H3</f>
+        <v>0.02</v>
+      </c>
+      <c r="E26" s="2">
+        <f>G13</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F26" s="2">
+        <f t="shared" si="3"/>
+        <v>6.123636363636363E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="2">
+        <f>H4</f>
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="E27" s="2">
+        <f>G13</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F27" s="2">
+        <f t="shared" si="3"/>
+        <v>5.6236363636363633E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E18:F18"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6D3A2C0-F7E4-44F1-9EB9-4625D672EE90}">
   <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3673,10 +4150,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="38"/>
+      <c r="B1" s="39"/>
       <c r="D1" s="17" t="s">
         <v>148</v>
       </c>
@@ -3788,10 +4265,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="39" t="s">
         <v>162</v>
       </c>
-      <c r="B13" s="38"/>
+      <c r="B13" s="39"/>
       <c r="D13" s="14"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -3868,10 +4345,10 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="38" t="s">
+      <c r="A24" s="39" t="s">
         <v>221</v>
       </c>
-      <c r="B24" s="38"/>
+      <c r="B24" s="39"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
@@ -4017,14 +4494,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="E1" s="39" t="s">
+      <c r="B1" s="39"/>
+      <c r="E1" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="F1" s="39"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
@@ -4102,10 +4579,10 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="B11" s="39"/>
+      <c r="B11" s="40"/>
       <c r="E11" s="15" t="s">
         <v>185</v>
       </c>
@@ -4538,10 +5015,10 @@
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="G8" s="28"/>
+      <c r="G8" s="29"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -4557,11 +5034,11 @@
         <f>D9*60</f>
         <v>60</v>
       </c>
-      <c r="F9" s="40">
+      <c r="F9" s="41">
         <f>C9/E9</f>
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="G9" s="40"/>
+      <c r="G9" s="41"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -4577,11 +5054,11 @@
         <f t="shared" ref="E10:E12" si="3">D10*60</f>
         <v>120</v>
       </c>
-      <c r="F10" s="40">
+      <c r="F10" s="41">
         <f t="shared" ref="F10" si="4">C10/E10</f>
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="G10" s="40"/>
+      <c r="G10" s="41"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -4597,11 +5074,11 @@
         <f t="shared" si="3"/>
         <v>300</v>
       </c>
-      <c r="F11" s="40">
+      <c r="F11" s="41">
         <f>C11/E11</f>
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="G11" s="40"/>
+      <c r="G11" s="41"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -4617,11 +5094,11 @@
         <f t="shared" si="3"/>
         <v>720</v>
       </c>
-      <c r="F12" s="40">
+      <c r="F12" s="41">
         <f>C12/E12</f>
         <v>6.6666666666666666E-2</v>
       </c>
-      <c r="G12" s="40"/>
+      <c r="G12" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4636,6 +5113,526 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ECA3B0D-3FD0-4ED6-A953-2417B5DF772B}">
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="30.7265625" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="17.08984375" customWidth="1"/>
+    <col min="5" max="5" width="22.26953125" customWidth="1"/>
+    <col min="6" max="6" width="25.36328125" customWidth="1"/>
+    <col min="7" max="7" width="19.54296875" customWidth="1"/>
+    <col min="8" max="8" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>8</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2">
+        <v>200</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>24</v>
+      </c>
+      <c r="C3">
+        <v>30</v>
+      </c>
+      <c r="D3">
+        <v>15</v>
+      </c>
+      <c r="E3">
+        <f>60*D3</f>
+        <v>900</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4">
+        <v>48</v>
+      </c>
+      <c r="C4">
+        <v>60</v>
+      </c>
+      <c r="D4">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E5" si="0">60*D4</f>
+        <v>1800</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>96</v>
+      </c>
+      <c r="C5">
+        <v>120</v>
+      </c>
+      <c r="D5">
+        <v>60</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>3600</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="29"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <f>D8*60</f>
+        <v>60</v>
+      </c>
+      <c r="F8" s="41">
+        <f>C8/E8</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="G8" s="41"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <f t="shared" ref="E9:E11" si="1">D9*60</f>
+        <v>120</v>
+      </c>
+      <c r="F9" s="41">
+        <f t="shared" ref="F9" si="2">C9/E9</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="G9" s="41"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10">
+        <v>20</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>300</v>
+      </c>
+      <c r="F10" s="41">
+        <f>C10/E10</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="G10" s="41"/>
+      <c r="H10" s="28"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11">
+        <v>48</v>
+      </c>
+      <c r="D11">
+        <v>12</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>720</v>
+      </c>
+      <c r="F11" s="41">
+        <f>C11/E11</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="G11" s="41"/>
+      <c r="H11" s="28"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15">
+        <v>13</v>
+      </c>
+      <c r="D15">
+        <v>100</v>
+      </c>
+      <c r="E15" s="43">
+        <f>C15/D15</f>
+        <v>0.13</v>
+      </c>
+      <c r="F15" s="43"/>
+      <c r="G15" s="28">
+        <f>E15*0.36</f>
+        <v>4.6800000000000001E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16">
+        <v>63.2</v>
+      </c>
+      <c r="D16">
+        <v>530</v>
+      </c>
+      <c r="E16" s="43">
+        <f t="shared" ref="E16:E22" si="3">C16/D16</f>
+        <v>0.11924528301886793</v>
+      </c>
+      <c r="F16" s="43"/>
+      <c r="G16" s="28">
+        <f t="shared" ref="G16:G22" si="4">E16*0.36</f>
+        <v>4.2928301886792454E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17">
+        <v>126</v>
+      </c>
+      <c r="D17">
+        <v>1100</v>
+      </c>
+      <c r="E17" s="43">
+        <f t="shared" si="3"/>
+        <v>0.11454545454545455</v>
+      </c>
+      <c r="F17" s="43"/>
+      <c r="G17" s="28">
+        <f t="shared" si="4"/>
+        <v>4.1236363636363634E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18">
+        <v>647</v>
+      </c>
+      <c r="D18">
+        <v>5950</v>
+      </c>
+      <c r="E18" s="43">
+        <f t="shared" si="3"/>
+        <v>0.10873949579831933</v>
+      </c>
+      <c r="F18" s="43"/>
+      <c r="G18" s="28">
+        <f t="shared" si="4"/>
+        <v>3.9146218487394961E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19">
+        <v>1313</v>
+      </c>
+      <c r="D19">
+        <v>12500</v>
+      </c>
+      <c r="E19" s="43">
+        <f t="shared" si="3"/>
+        <v>0.10503999999999999</v>
+      </c>
+      <c r="F19" s="43"/>
+      <c r="G19" s="28">
+        <f t="shared" si="4"/>
+        <v>3.7814399999999998E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20">
+        <v>2528</v>
+      </c>
+      <c r="D20">
+        <v>25000</v>
+      </c>
+      <c r="E20" s="43">
+        <f t="shared" si="3"/>
+        <v>0.10112</v>
+      </c>
+      <c r="F20" s="43"/>
+      <c r="G20" s="28">
+        <f t="shared" si="4"/>
+        <v>3.6403199999999997E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21">
+        <v>6641</v>
+      </c>
+      <c r="D21">
+        <v>67500</v>
+      </c>
+      <c r="E21" s="43">
+        <f t="shared" si="3"/>
+        <v>9.8385185185185187E-2</v>
+      </c>
+      <c r="F21" s="43"/>
+      <c r="G21" s="28">
+        <f t="shared" si="4"/>
+        <v>3.5418666666666668E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22">
+        <v>13584</v>
+      </c>
+      <c r="D22">
+        <v>142800</v>
+      </c>
+      <c r="E22" s="43">
+        <f t="shared" si="3"/>
+        <v>9.5126050420168071E-2</v>
+      </c>
+      <c r="F22" s="43"/>
+      <c r="G22" s="28">
+        <f t="shared" si="4"/>
+        <v>3.4245378151260504E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="2" t="e">
+        <f>#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="E28" s="2">
+        <f>G17</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F28" s="2" t="e">
+        <f>D28+E28</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" t="s">
+        <v>54</v>
+      </c>
+      <c r="D29" s="2" t="e">
+        <f>#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="E29" s="2">
+        <f>G17</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F29" s="2" t="e">
+        <f t="shared" ref="F29:F31" si="5">D29+E29</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="2">
+        <f>H3</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="2">
+        <f>G17</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F30" s="2">
+        <f t="shared" si="5"/>
+        <v>4.1236363636363634E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="2">
+        <f>H4</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="2">
+        <f>G17</f>
+        <v>4.1236363636363634E-2</v>
+      </c>
+      <c r="F31" s="2">
+        <f t="shared" si="5"/>
+        <v>4.1236363636363634E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E17:F17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C29AEF30-3233-4363-A39E-B6F27417D9E0}">
   <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4835,10 +5832,10 @@
       <c r="A10" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="41" t="s">
+      <c r="G10" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="41"/>
+      <c r="H10" s="42"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -4854,11 +5851,11 @@
         <f>C11/D11</f>
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="G11" s="40">
+      <c r="G11" s="41">
         <f>F11*100</f>
         <v>0.03</v>
       </c>
-      <c r="H11" s="40"/>
+      <c r="H11" s="41"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -4874,11 +5871,11 @@
         <f t="shared" ref="F12:F14" si="4">C12/D12</f>
         <v>2.3999999999999998E-4</v>
       </c>
-      <c r="G12" s="40">
+      <c r="G12" s="41">
         <f t="shared" ref="G12:G14" si="5">F12*100</f>
         <v>2.3999999999999997E-2</v>
       </c>
-      <c r="H12" s="40"/>
+      <c r="H12" s="41"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -4894,11 +5891,11 @@
         <f t="shared" si="4"/>
         <v>1.7999999999999998E-4</v>
       </c>
-      <c r="G13" s="40">
+      <c r="G13" s="41">
         <f t="shared" si="5"/>
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="H13" s="40"/>
+      <c r="H13" s="41"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -4914,11 +5911,11 @@
         <f t="shared" si="4"/>
         <v>1E-4</v>
       </c>
-      <c r="G14" s="40">
+      <c r="G14" s="41">
         <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
-      <c r="H14" s="40"/>
+      <c r="H14" s="41"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -4947,7 +5944,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7DDD1A3-7BAD-4063-B1C6-8CB7B009FF65}">
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5045,16 +6042,16 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5066,7 +6063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{872691C0-4F1A-478B-990A-02E553FB2165}">
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5243,12 +6240,12 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I14" s="40"/>
-      <c r="J14" s="40"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="41"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I15" s="40"/>
-      <c r="J15" s="40"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -5267,471 +6264,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31193713-3E89-4A71-A172-6D7922B9768D}">
-  <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="15.1796875" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="17.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" customWidth="1"/>
-    <col min="6" max="6" width="25.36328125" customWidth="1"/>
-    <col min="7" max="7" width="19.54296875" customWidth="1"/>
-    <col min="8" max="8" width="21" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>50</v>
-      </c>
-      <c r="E2">
-        <f>B2/D2</f>
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <f>C2/D2</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="2">
-        <f>E2*100</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="2">
-        <f>F2*100</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3">
-        <v>96</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-      <c r="D3">
-        <v>2500</v>
-      </c>
-      <c r="E3">
-        <f>B3/(D3*12)</f>
-        <v>3.2000000000000002E-3</v>
-      </c>
-      <c r="F3">
-        <f>C3/D3</f>
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="G3" s="2">
-        <f>E3*5</f>
-        <v>1.6E-2</v>
-      </c>
-      <c r="H3" s="2">
-        <f>F3*5</f>
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4">
-        <v>288</v>
-      </c>
-      <c r="C4">
-        <v>30</v>
-      </c>
-      <c r="D4">
-        <v>10000</v>
-      </c>
-      <c r="E4">
-        <f>B4/(D4*12)</f>
-        <v>2.3999999999999998E-3</v>
-      </c>
-      <c r="F4">
-        <f t="shared" ref="F4" si="0">C4/D4</f>
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="G4" s="2">
-        <f>E4*5</f>
-        <v>1.1999999999999999E-2</v>
-      </c>
-      <c r="H4" s="2">
-        <f>F4*5</f>
-        <v>1.4999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11">
-        <v>13</v>
-      </c>
-      <c r="D11">
-        <v>100</v>
-      </c>
-      <c r="E11" s="42">
-        <f t="shared" ref="E11:E18" si="1">C11/D11</f>
-        <v>0.13</v>
-      </c>
-      <c r="F11" s="42"/>
-      <c r="G11" s="40">
-        <f>E11*0.36</f>
-        <v>4.6800000000000001E-2</v>
-      </c>
-      <c r="H11" s="40"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12">
-        <v>63.2</v>
-      </c>
-      <c r="D12">
-        <v>530</v>
-      </c>
-      <c r="E12" s="42">
-        <f t="shared" si="1"/>
-        <v>0.11924528301886793</v>
-      </c>
-      <c r="F12" s="42"/>
-      <c r="G12" s="40">
-        <f t="shared" ref="G12:G18" si="2">E12*0.36</f>
-        <v>4.2928301886792454E-2</v>
-      </c>
-      <c r="H12" s="40"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13">
-        <v>126</v>
-      </c>
-      <c r="D13">
-        <v>1100</v>
-      </c>
-      <c r="E13" s="42">
-        <f t="shared" si="1"/>
-        <v>0.11454545454545455</v>
-      </c>
-      <c r="F13" s="42"/>
-      <c r="G13" s="40">
-        <f t="shared" si="2"/>
-        <v>4.1236363636363634E-2</v>
-      </c>
-      <c r="H13" s="40"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14">
-        <v>647</v>
-      </c>
-      <c r="D14">
-        <v>5950</v>
-      </c>
-      <c r="E14" s="42">
-        <f t="shared" si="1"/>
-        <v>0.10873949579831933</v>
-      </c>
-      <c r="F14" s="42"/>
-      <c r="G14" s="40">
-        <f t="shared" si="2"/>
-        <v>3.9146218487394961E-2</v>
-      </c>
-      <c r="H14" s="40"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15">
-        <v>1313</v>
-      </c>
-      <c r="D15">
-        <v>12500</v>
-      </c>
-      <c r="E15" s="42">
-        <f t="shared" si="1"/>
-        <v>0.10503999999999999</v>
-      </c>
-      <c r="F15" s="42"/>
-      <c r="G15" s="40">
-        <f t="shared" si="2"/>
-        <v>3.7814399999999998E-2</v>
-      </c>
-      <c r="H15" s="40"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16">
-        <v>2528</v>
-      </c>
-      <c r="D16">
-        <v>25000</v>
-      </c>
-      <c r="E16" s="42">
-        <f t="shared" si="1"/>
-        <v>0.10112</v>
-      </c>
-      <c r="F16" s="42"/>
-      <c r="G16" s="40">
-        <f t="shared" si="2"/>
-        <v>3.6403199999999997E-2</v>
-      </c>
-      <c r="H16" s="40"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17">
-        <v>6641</v>
-      </c>
-      <c r="D17">
-        <v>67500</v>
-      </c>
-      <c r="E17" s="42">
-        <f t="shared" si="1"/>
-        <v>9.8385185185185187E-2</v>
-      </c>
-      <c r="F17" s="42"/>
-      <c r="G17" s="40">
-        <f t="shared" si="2"/>
-        <v>3.5418666666666668E-2</v>
-      </c>
-      <c r="H17" s="40"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18">
-        <v>13584</v>
-      </c>
-      <c r="D18">
-        <v>142800</v>
-      </c>
-      <c r="E18" s="42">
-        <f t="shared" si="1"/>
-        <v>9.5126050420168071E-2</v>
-      </c>
-      <c r="F18" s="42"/>
-      <c r="G18" s="40">
-        <f t="shared" si="2"/>
-        <v>3.4245378151260504E-2</v>
-      </c>
-      <c r="H18" s="40"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>61</v>
-      </c>
-      <c r="B24" t="s">
-        <v>37</v>
-      </c>
-      <c r="C24" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="2">
-        <f>G3</f>
-        <v>1.6E-2</v>
-      </c>
-      <c r="E24" s="2">
-        <f>G13</f>
-        <v>4.1236363636363634E-2</v>
-      </c>
-      <c r="F24" s="2">
-        <f>D24+E24</f>
-        <v>5.7236363636363634E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>61</v>
-      </c>
-      <c r="B25" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" t="s">
-        <v>54</v>
-      </c>
-      <c r="D25" s="2">
-        <f>G4</f>
-        <v>1.1999999999999999E-2</v>
-      </c>
-      <c r="E25" s="2">
-        <f>G13</f>
-        <v>4.1236363636363634E-2</v>
-      </c>
-      <c r="F25" s="2">
-        <f t="shared" ref="F25:F27" si="3">D25+E25</f>
-        <v>5.323636363636363E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" t="s">
-        <v>38</v>
-      </c>
-      <c r="C26" t="s">
-        <v>14</v>
-      </c>
-      <c r="D26" s="2">
-        <f>H3</f>
-        <v>0.02</v>
-      </c>
-      <c r="E26" s="2">
-        <f>G13</f>
-        <v>4.1236363636363634E-2</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" si="3"/>
-        <v>6.123636363636363E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>60</v>
-      </c>
-      <c r="B27" t="s">
-        <v>38</v>
-      </c>
-      <c r="C27" t="s">
-        <v>54</v>
-      </c>
-      <c r="D27" s="2">
-        <f>H4</f>
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="E27" s="2">
-        <f>G13</f>
-        <v>4.1236363636363634E-2</v>
-      </c>
-      <c r="F27" s="2">
-        <f t="shared" si="3"/>
-        <v>5.6236363636363633E-2</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E14:F14"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>